<commit_message>
PMO: Phase 1 platform Approved — refresh board status.
Mark G-24–G-28, G-01, G-03, G-16 Done; T+8 PoC in progress; B2C post-launch.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/DigiThane_Kickoff_RACI_TMC.xlsx
+++ b/public/DigiThane_Kickoff_RACI_TMC.xlsx
@@ -445,6 +445,18 @@
     <t>Web Engineer, Analytics Engineer</t>
   </si>
   <si>
+    <t>G-03</t>
+  </si>
+  <si>
+    <t>News, notices, and editable policy text</t>
+  </si>
+  <si>
+    <t>Backend Engineer, Web Engineer</t>
+  </si>
+  <si>
+    <t>9 Oct 2026</t>
+  </si>
+  <si>
     <t>T+8</t>
   </si>
   <si>
@@ -454,18 +466,6 @@
     <t>Chief Technology Officer</t>
   </si>
   <si>
-    <t>G-03</t>
-  </si>
-  <si>
-    <t>News, notices, and editable policy text</t>
-  </si>
-  <si>
-    <t>Backend Engineer, Web Engineer</t>
-  </si>
-  <si>
-    <t>9 Oct 2026</t>
-  </si>
-  <si>
     <t>2 Services</t>
   </si>
   <si>
@@ -850,7 +850,7 @@
     <t>T+8 Proof of concept</t>
   </si>
   <si>
-    <t>Login, home, master control centre. Screen prototypes already done.</t>
+    <t>Login, home, search, CMS notices, master control centre — Phase 1 platform Approved 13 Sep 2026.</t>
   </si>
   <si>
     <t>B2C pack</t>
@@ -859,7 +859,7 @@
     <t>After MCC → UAT</t>
   </si>
   <si>
-    <t>One stream: merchants, marketplace, ads, offers, classifieds, events, jobs, halls, premium, parking, property, tourism, clinics, deals.</t>
+    <t>Post-launch for TMC clock (AD-039). One stream: merchants, marketplace, ads, offers, classifieds, events, jobs, halls, premium, parking, property, tourism, clinics, deals.</t>
   </si>
   <si>
     <t>UAT 1</t>
@@ -3281,7 +3281,7 @@
         <v>143</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -3289,16 +3289,16 @@
         <v>113</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3499,7 +3499,7 @@
         <v>182</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E26" s="23" t="s">
         <v>162</v>
@@ -3712,7 +3712,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>221</v>

</xml_diff>